<commit_message>
Improved results after update of bounding box sizing
</commit_message>
<xml_diff>
--- a/results/01_pre_QA_QC_transcribed_hydroclimate_data/203/203_196905_SF.JPG_pre_QA_QC.xlsx
+++ b/results/01_pre_QA_QC_transcribed_hydroclimate_data/203/203_196905_SF.JPG_pre_QA_QC.xlsx
@@ -679,7 +679,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1362
+          <t xml:space="preserve">1862
 </t>
         </is>
       </c>
@@ -697,13 +697,13 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">245
+          <t xml:space="preserve">243
 </t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">817
+          <t xml:space="preserve">872
 </t>
         </is>
       </c>
@@ -715,7 +715,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">17
+          <t xml:space="preserve">118
 </t>
         </is>
       </c>
@@ -763,7 +763,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">288
+          <t xml:space="preserve">287
 </t>
         </is>
       </c>
@@ -775,7 +775,7 @@
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">221
+          <t xml:space="preserve">271
 </t>
         </is>
       </c>
@@ -799,7 +799,7 @@
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">828
+          <t xml:space="preserve">228
 </t>
         </is>
       </c>
@@ -811,7 +811,7 @@
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1818
+          <t xml:space="preserve">818
 </t>
         </is>
       </c>
@@ -838,13 +838,13 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2038
+          <t xml:space="preserve">4038
 </t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8326
+          <t xml:space="preserve">326
 </t>
         </is>
       </c>
@@ -886,7 +886,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">010
+          <t xml:space="preserve">00
 </t>
         </is>
       </c>
@@ -910,7 +910,7 @@
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9090
+          <t xml:space="preserve">990
 </t>
         </is>
       </c>
@@ -964,13 +964,13 @@
       </c>
       <c r="X5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2728
+          <t xml:space="preserve">278
 </t>
         </is>
       </c>
       <c r="Y5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1411
+          <t xml:space="preserve">71740
 </t>
         </is>
       </c>
@@ -997,7 +997,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1223
+          <t xml:space="preserve">4223
 </t>
         </is>
       </c>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">122
+          <t xml:space="preserve">288
 </t>
         </is>
       </c>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">21846
+          <t xml:space="preserve">1152
 </t>
         </is>
       </c>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0800
+          <t xml:space="preserve">00
 </t>
         </is>
       </c>
@@ -1099,25 +1099,25 @@
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">228
+          <t xml:space="preserve">928
 </t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">204
+          <t xml:space="preserve">207
 </t>
         </is>
       </c>
       <c r="V6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">282
+          <t xml:space="preserve">281
 </t>
         </is>
       </c>
       <c r="W6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2317
+          <t xml:space="preserve">237
 </t>
         </is>
       </c>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="Y6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">166141
+          <t xml:space="preserve">664
 </t>
         </is>
       </c>
@@ -1156,25 +1156,25 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">64725
+          <t xml:space="preserve">4725
 </t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">347
+          <t xml:space="preserve">348
 </t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1199
+          <t xml:space="preserve">193
 </t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">210
+          <t xml:space="preserve">2720
 </t>
         </is>
       </c>
@@ -1192,13 +1192,13 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">479
+          <t xml:space="preserve">847
 </t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">19
+          <t xml:space="preserve">79
 </t>
         </is>
       </c>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="R7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">222
+          <t xml:space="preserve">22
 </t>
         </is>
       </c>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="V7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1295
+          <t xml:space="preserve">295
 </t>
         </is>
       </c>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="Z7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">158
+          <t xml:space="preserve">138
 </t>
         </is>
       </c>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">160
+          <t xml:space="preserve">140
 </t>
         </is>
       </c>
@@ -1387,7 +1387,7 @@
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">965
+          <t xml:space="preserve">2965
 </t>
         </is>
       </c>
@@ -1447,7 +1447,7 @@
       </c>
       <c r="Y8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">914
+          <t xml:space="preserve">974
 </t>
         </is>
       </c>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">17812
+          <t xml:space="preserve">17832
 </t>
         </is>
       </c>
@@ -1492,13 +1492,13 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">130 17
+          <t xml:space="preserve">230 8
 </t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">659
+          <t xml:space="preserve">679
 </t>
         </is>
       </c>
@@ -1510,13 +1510,13 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">166
+          <t xml:space="preserve">168
 </t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">128
+          <t xml:space="preserve">275
 </t>
         </is>
       </c>
@@ -1546,31 +1546,31 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8942
+          <t xml:space="preserve">4942
 </t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">82
+          <t xml:space="preserve">112
 </t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11796
+          <t xml:space="preserve">1496
 </t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1229
+          <t xml:space="preserve">1219
 </t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1551
+          <t xml:space="preserve">1357
 </t>
         </is>
       </c>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="U9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">810
+          <t xml:space="preserve">820
 </t>
         </is>
       </c>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="W9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11168
+          <t xml:space="preserve">1168
 </t>
         </is>
       </c>
@@ -1606,13 +1606,13 @@
       </c>
       <c r="Y9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3888
+          <t xml:space="preserve">37888
 </t>
         </is>
       </c>
       <c r="Z9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1416
+          <t xml:space="preserve">416
 </t>
         </is>
       </c>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">81885
+          <t xml:space="preserve">354
 </t>
         </is>
       </c>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">194
+          <t xml:space="preserve">198
 </t>
         </is>
       </c>
@@ -1663,7 +1663,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">119
+          <t xml:space="preserve">179
 </t>
         </is>
       </c>
@@ -1675,12 +1675,15 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">29
-</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="n">
-        <v/>
+          <t xml:space="preserve">55
+</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11 1
+</t>
+        </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
@@ -1714,19 +1717,19 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">299
+          <t xml:space="preserve">1299
 </t>
         </is>
       </c>
       <c r="R10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">944
+          <t xml:space="preserve">244
 </t>
         </is>
       </c>
       <c r="S10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">278
+          <t xml:space="preserve">271
 </t>
         </is>
       </c>
@@ -1756,7 +1759,7 @@
       </c>
       <c r="X10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8162
+          <t xml:space="preserve">267
 </t>
         </is>
       </c>
@@ -1768,7 +1771,7 @@
       </c>
       <c r="Z10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">183
+          <t xml:space="preserve">83
 </t>
         </is>
       </c>
@@ -1789,7 +1792,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12656
+          <t xml:space="preserve">2656
 </t>
         </is>
       </c>
@@ -1825,7 +1828,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">16
+          <t xml:space="preserve">06
 </t>
         </is>
       </c>
@@ -1855,13 +1858,13 @@
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">243
+          <t xml:space="preserve">245
 </t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9273
+          <t xml:space="preserve">213
 </t>
         </is>
       </c>
@@ -1879,19 +1882,19 @@
       </c>
       <c r="R11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">255
+          <t xml:space="preserve">235
 </t>
         </is>
       </c>
       <c r="S11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9298
+          <t xml:space="preserve">298
 </t>
         </is>
       </c>
       <c r="T11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">7206
+          <t xml:space="preserve">706
 </t>
         </is>
       </c>
@@ -1903,13 +1906,13 @@
       </c>
       <c r="V11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2721
+          <t xml:space="preserve">271
 </t>
         </is>
       </c>
       <c r="W11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9169
+          <t xml:space="preserve">949
 </t>
         </is>
       </c>
@@ -1921,13 +1924,13 @@
       </c>
       <c r="Y11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">28940
+          <t xml:space="preserve">8940
 </t>
         </is>
       </c>
       <c r="Z11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">118
+          <t xml:space="preserve">58
 </t>
         </is>
       </c>
@@ -1948,13 +1951,13 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3471
+          <t xml:space="preserve">2421
 </t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">918
+          <t xml:space="preserve">818
 </t>
         </is>
       </c>
@@ -1984,7 +1987,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12271
+          <t xml:space="preserve">27
 </t>
         </is>
       </c>
@@ -2008,18 +2011,19 @@
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>93505</t>
+          <t xml:space="preserve">230
+</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2179
+          <t xml:space="preserve">279
 </t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">974
+          <t xml:space="preserve">9275
 </t>
         </is>
       </c>
@@ -2043,13 +2047,13 @@
       </c>
       <c r="S12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">211
+          <t xml:space="preserve">271
 </t>
         </is>
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">518
+          <t xml:space="preserve">598
 </t>
         </is>
       </c>
@@ -2085,7 +2089,7 @@
       </c>
       <c r="Z12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">216
+          <t xml:space="preserve">817
 </t>
         </is>
       </c>
@@ -2124,7 +2128,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">866
+          <t xml:space="preserve">266
 </t>
         </is>
       </c>
@@ -2142,13 +2146,13 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">183
+          <t xml:space="preserve">33
 </t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">60
+          <t xml:space="preserve">160
 </t>
         </is>
       </c>
@@ -2202,13 +2206,13 @@
       </c>
       <c r="S13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1218
+          <t xml:space="preserve">258
 </t>
         </is>
       </c>
       <c r="T13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4274
+          <t xml:space="preserve">527
 </t>
         </is>
       </c>
@@ -2232,7 +2236,7 @@
       </c>
       <c r="X13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">295
+          <t xml:space="preserve">293
 </t>
         </is>
       </c>
@@ -2271,7 +2275,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">307
+          <t xml:space="preserve">3071
 </t>
         </is>
       </c>
@@ -2301,108 +2305,108 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">15
+          <t xml:space="preserve">115
 </t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">21
-</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="n">
+          <t xml:space="preserve">821
+</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">111
+</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">224
+</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">221
+</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">264
+</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">973
+</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07
+</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">824
+</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">211
+</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">242
+</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">890
+</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">29
+</t>
+        </is>
+      </c>
+      <c r="V14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">220
+</t>
+        </is>
+      </c>
+      <c r="W14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">216
+</t>
+        </is>
+      </c>
+      <c r="X14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">255
+</t>
+        </is>
+      </c>
+      <c r="Y14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">960
+</t>
+        </is>
+      </c>
+      <c r="Z14" s="3" t="n">
         <v/>
-      </c>
-      <c r="L14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">224
-</t>
-        </is>
-      </c>
-      <c r="M14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">221
-</t>
-        </is>
-      </c>
-      <c r="N14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">264
-</t>
-        </is>
-      </c>
-      <c r="O14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">973
-</t>
-        </is>
-      </c>
-      <c r="P14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">07
-</t>
-        </is>
-      </c>
-      <c r="Q14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">824
-</t>
-        </is>
-      </c>
-      <c r="R14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">211
-</t>
-        </is>
-      </c>
-      <c r="S14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">242
-</t>
-        </is>
-      </c>
-      <c r="T14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">890
-</t>
-        </is>
-      </c>
-      <c r="U14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">29
-</t>
-        </is>
-      </c>
-      <c r="V14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">220
-</t>
-        </is>
-      </c>
-      <c r="W14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12116
-</t>
-        </is>
-      </c>
-      <c r="X14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">255
-</t>
-        </is>
-      </c>
-      <c r="Y14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">960
-</t>
-        </is>
-      </c>
-      <c r="Z14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">109
-</t>
-        </is>
       </c>
       <c r="AA14" s="3" t="inlineStr">
         <is>
@@ -2421,7 +2425,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2828
+          <t xml:space="preserve">3596
 </t>
         </is>
       </c>
@@ -2457,7 +2461,7 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">84
+          <t xml:space="preserve">24
 </t>
         </is>
       </c>
@@ -2469,7 +2473,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2517
+          <t xml:space="preserve">237
 </t>
         </is>
       </c>
@@ -2481,7 +2485,7 @@
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1216
+          <t xml:space="preserve">216
 </t>
         </is>
       </c>
@@ -2493,13 +2497,13 @@
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1000
+          <t xml:space="preserve">1002
 </t>
         </is>
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">80
+          <t xml:space="preserve">00
 </t>
         </is>
       </c>
@@ -2553,13 +2557,13 @@
       </c>
       <c r="Y15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">7381
+          <t xml:space="preserve">731
 </t>
         </is>
       </c>
       <c r="Z15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1006
+          <t xml:space="preserve">106
 </t>
         </is>
       </c>
@@ -2580,7 +2584,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12912
+          <t xml:space="preserve">12212
 </t>
         </is>
       </c>
@@ -2592,13 +2596,12 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1055
-</t>
+          <t>12551</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1514
+          <t xml:space="preserve">1319
 </t>
         </is>
       </c>
@@ -2634,13 +2637,13 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11106
+          <t xml:space="preserve">1106
 </t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1095
+          <t xml:space="preserve">1098
 </t>
         </is>
       </c>
@@ -2652,7 +2655,7 @@
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">24901
+          <t xml:space="preserve">14901
 </t>
         </is>
       </c>
@@ -2670,13 +2673,13 @@
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1219
+          <t xml:space="preserve">12219
 </t>
         </is>
       </c>
       <c r="S16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11362
+          <t xml:space="preserve">11361
 </t>
         </is>
       </c>
@@ -2745,7 +2748,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">816
+          <t xml:space="preserve">316
 </t>
         </is>
       </c>
@@ -2775,7 +2778,7 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">123
+          <t xml:space="preserve">23
 </t>
         </is>
       </c>
@@ -2787,7 +2790,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11
+          <t xml:space="preserve">0060
 </t>
         </is>
       </c>
@@ -2811,7 +2814,7 @@
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3980
+          <t xml:space="preserve">9280
 </t>
         </is>
       </c>
@@ -2823,7 +2826,7 @@
       </c>
       <c r="Q17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">291
+          <t xml:space="preserve">297
 </t>
         </is>
       </c>
@@ -2847,24 +2850,24 @@
       </c>
       <c r="U17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">158
+          <t xml:space="preserve">153
 </t>
         </is>
       </c>
       <c r="V17" s="3" t="inlineStr">
         <is>
-          <t>063</t>
+          <t>83</t>
         </is>
       </c>
       <c r="W17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2141
+          <t xml:space="preserve">241
 </t>
         </is>
       </c>
       <c r="X17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2846
+          <t xml:space="preserve">285
 </t>
         </is>
       </c>
@@ -2903,7 +2906,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">821
+          <t xml:space="preserve">321
 </t>
         </is>
       </c>
@@ -2915,15 +2918,12 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9861
-</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">109
-</t>
-        </is>
+          <t xml:space="preserve">261
+</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v/>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
@@ -2939,13 +2939,13 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">43
+          <t xml:space="preserve">143
 </t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1064
+          <t xml:space="preserve">104
 </t>
         </is>
       </c>
@@ -2963,13 +2963,13 @@
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2128
+          <t xml:space="preserve">248
 </t>
         </is>
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">913
+          <t xml:space="preserve">973
 </t>
         </is>
       </c>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="R18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1252
+          <t xml:space="preserve">252
 </t>
         </is>
       </c>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">280
+          <t xml:space="preserve">380
 </t>
         </is>
       </c>
@@ -3029,13 +3029,13 @@
       </c>
       <c r="Y18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">714
+          <t xml:space="preserve">719
 </t>
         </is>
       </c>
       <c r="Z18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1110
+          <t xml:space="preserve">110
 </t>
         </is>
       </c>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">214
+          <t xml:space="preserve">2914
 </t>
         </is>
       </c>
@@ -3134,13 +3134,13 @@
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">806
+          <t xml:space="preserve">106
 </t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8299
+          <t xml:space="preserve">0299
 </t>
         </is>
       </c>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="S19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">511
+          <t xml:space="preserve">311
 </t>
         </is>
       </c>
@@ -3170,31 +3170,31 @@
       </c>
       <c r="V19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2163
+          <t xml:space="preserve">243
 </t>
         </is>
       </c>
       <c r="W19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12898
+          <t xml:space="preserve">1289
 </t>
         </is>
       </c>
       <c r="X19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">241
+          <t xml:space="preserve">271
 </t>
         </is>
       </c>
       <c r="Y19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8290
+          <t xml:space="preserve">890
 </t>
         </is>
       </c>
       <c r="Z19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1859
+          <t xml:space="preserve">83
 </t>
         </is>
       </c>
@@ -3215,7 +3215,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">38659
+          <t xml:space="preserve">3659
 </t>
         </is>
       </c>
@@ -3227,13 +3227,13 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">215
+          <t xml:space="preserve">2185
 </t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2081
+          <t xml:space="preserve">285
 </t>
         </is>
       </c>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">125
+          <t xml:space="preserve">25
 </t>
         </is>
       </c>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">100
+          <t xml:space="preserve">00
 </t>
         </is>
       </c>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9280
+          <t xml:space="preserve">980
 </t>
         </is>
       </c>
@@ -3299,7 +3299,7 @@
       </c>
       <c r="Q20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">209
+          <t xml:space="preserve">307
 </t>
         </is>
       </c>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="S20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">275
+          <t xml:space="preserve">2175
 </t>
         </is>
       </c>
@@ -3335,25 +3335,25 @@
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1288
+          <t xml:space="preserve">228
 </t>
         </is>
       </c>
       <c r="X20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">212
+          <t xml:space="preserve">272
 </t>
         </is>
       </c>
       <c r="Y20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1250
+          <t xml:space="preserve">7250
 </t>
         </is>
       </c>
       <c r="Z20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">191
+          <t xml:space="preserve">91
 </t>
         </is>
       </c>
@@ -3380,7 +3380,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">307
+          <t xml:space="preserve">3072
 </t>
         </is>
       </c>
@@ -3434,13 +3434,13 @@
       </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">219
+          <t xml:space="preserve">215
 </t>
         </is>
       </c>
       <c r="N21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">236
+          <t xml:space="preserve">256
 </t>
         </is>
       </c>
@@ -3470,7 +3470,7 @@
       </c>
       <c r="S21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">912
+          <t xml:space="preserve">312
 </t>
         </is>
       </c>
@@ -3494,7 +3494,7 @@
       </c>
       <c r="W21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2466
+          <t xml:space="preserve">2266
 </t>
         </is>
       </c>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="Y21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">7123
+          <t xml:space="preserve">723
 </t>
         </is>
       </c>
@@ -3557,7 +3557,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">128
+          <t xml:space="preserve">118
 </t>
         </is>
       </c>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">29
+          <t xml:space="preserve">27
 </t>
         </is>
       </c>
@@ -3593,7 +3593,7 @@
       </c>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">220
+          <t xml:space="preserve">210
 </t>
         </is>
       </c>
@@ -3623,7 +3623,7 @@
       </c>
       <c r="R22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">259
+          <t xml:space="preserve">299
 </t>
         </is>
       </c>
@@ -3641,13 +3641,13 @@
       </c>
       <c r="U22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">152
+          <t xml:space="preserve">192
 </t>
         </is>
       </c>
       <c r="V22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">865
+          <t xml:space="preserve">8265
 </t>
         </is>
       </c>
@@ -3659,7 +3659,7 @@
       </c>
       <c r="X22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1294
+          <t xml:space="preserve">297
 </t>
         </is>
       </c>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="Z22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12449
+          <t xml:space="preserve">1449
 </t>
         </is>
       </c>
@@ -3692,30 +3692,30 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>85196</t>
+          <t xml:space="preserve">17396
+</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">14685
+          <t xml:space="preserve">1675
 </t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">10742
+          <t xml:space="preserve">1072
 </t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1324
-</t>
+          <t>1388</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">503
+          <t xml:space="preserve">203
 </t>
         </is>
       </c>
@@ -3733,12 +3733,12 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>1045</t>
+          <t>104</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>4951</t>
+          <t>491</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">15657
+          <t xml:space="preserve">1557
 </t>
         </is>
       </c>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="T23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">33251
+          <t xml:space="preserve">3251
 </t>
         </is>
       </c>
@@ -3803,13 +3803,13 @@
       </c>
       <c r="V23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1384
+          <t xml:space="preserve">1344
 </t>
         </is>
       </c>
       <c r="W23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1203
+          <t xml:space="preserve">0203
 </t>
         </is>
       </c>
@@ -3827,8 +3827,7 @@
       </c>
       <c r="Z23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">921
-</t>
+          <t>3625</t>
         </is>
       </c>
       <c r="AA23" s="3" t="inlineStr">
@@ -3848,7 +3847,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>3439</t>
+          <t>3432</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -3865,7 +3864,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">265
+          <t xml:space="preserve">263
 </t>
         </is>
       </c>
@@ -3883,7 +3882,7 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">122
+          <t xml:space="preserve">22
 </t>
         </is>
       </c>
@@ -3895,7 +3894,7 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11
+          <t xml:space="preserve">1
 </t>
         </is>
       </c>
@@ -3937,13 +3936,13 @@
       </c>
       <c r="R24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">256
+          <t xml:space="preserve">856
 </t>
         </is>
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">894
+          <t xml:space="preserve">294
 </t>
         </is>
       </c>
@@ -3973,19 +3972,18 @@
       </c>
       <c r="X24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1292
+          <t xml:space="preserve">232
 </t>
         </is>
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">798
-</t>
+          <t>29813</t>
         </is>
       </c>
       <c r="Z24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">83
+          <t xml:space="preserve">73
 </t>
         </is>
       </c>
@@ -4024,13 +4022,13 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">239
+          <t xml:space="preserve">235
 </t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">86
+          <t xml:space="preserve">57
 </t>
         </is>
       </c>
@@ -4054,7 +4052,7 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">234
+          <t xml:space="preserve">237
 </t>
         </is>
       </c>
@@ -4078,7 +4076,7 @@
       </c>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9140
+          <t xml:space="preserve">970
 </t>
         </is>
       </c>
@@ -4096,7 +4094,7 @@
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">841
+          <t xml:space="preserve">241
 </t>
         </is>
       </c>
@@ -4114,12 +4112,15 @@
       </c>
       <c r="U25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">215
-</t>
-        </is>
-      </c>
-      <c r="V25" s="3" t="n">
-        <v/>
+          <t xml:space="preserve">53
+</t>
+        </is>
+      </c>
+      <c r="V25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2144
+</t>
+        </is>
       </c>
       <c r="W25" s="3" t="inlineStr">
         <is>
@@ -4129,13 +4130,13 @@
       </c>
       <c r="X25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1268
+          <t xml:space="preserve">268
 </t>
         </is>
       </c>
       <c r="Y25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">84174
+          <t xml:space="preserve">87817
 </t>
         </is>
       </c>
@@ -4171,7 +4172,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">240
+          <t xml:space="preserve">210
 </t>
         </is>
       </c>
@@ -4183,7 +4184,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">121
+          <t xml:space="preserve">141
 </t>
         </is>
       </c>
@@ -4195,13 +4196,13 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">899
+          <t xml:space="preserve">09
 </t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">041
+          <t xml:space="preserve">07
 </t>
         </is>
       </c>
@@ -4225,7 +4226,7 @@
       </c>
       <c r="N26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">259
+          <t xml:space="preserve">255
 </t>
         </is>
       </c>
@@ -4249,7 +4250,7 @@
       </c>
       <c r="R26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">235
+          <t xml:space="preserve">233
 </t>
         </is>
       </c>
@@ -4261,7 +4262,7 @@
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">920
+          <t xml:space="preserve">1920
 </t>
         </is>
       </c>
@@ -4285,7 +4286,7 @@
       </c>
       <c r="X26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2711
+          <t xml:space="preserve">271
 </t>
         </is>
       </c>
@@ -4297,7 +4298,7 @@
       </c>
       <c r="Z26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1245
+          <t xml:space="preserve">24
 </t>
         </is>
       </c>
@@ -4324,7 +4325,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>305</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -4335,8 +4336,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">854
-</t>
+          <t>255</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>503</t>
+          <t>504</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
@@ -4406,7 +4406,7 @@
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2169
+          <t xml:space="preserve">249
 </t>
         </is>
       </c>
@@ -4430,19 +4430,19 @@
       </c>
       <c r="V27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">869
+          <t xml:space="preserve">28269
 </t>
         </is>
       </c>
       <c r="W27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">944
+          <t xml:space="preserve">244
 </t>
         </is>
       </c>
       <c r="X27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12890
+          <t xml:space="preserve">2890
 </t>
         </is>
       </c>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="Z27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">124
+          <t xml:space="preserve">64
 </t>
         </is>
       </c>
@@ -4481,7 +4481,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5918
+          <t xml:space="preserve">318
 </t>
         </is>
       </c>
@@ -4547,13 +4547,13 @@
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">973
+          <t xml:space="preserve">97
 </t>
         </is>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">08
+          <t xml:space="preserve">18
 </t>
         </is>
       </c>
@@ -4613,7 +4613,7 @@
       </c>
       <c r="Z28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1074
+          <t xml:space="preserve">107
 </t>
         </is>
       </c>
@@ -4640,19 +4640,19 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3165
+          <t xml:space="preserve">315
 </t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">205
+          <t xml:space="preserve">20805
 </t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">960
+          <t xml:space="preserve">260
 </t>
         </is>
       </c>
@@ -4676,7 +4676,7 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">126
+          <t xml:space="preserve">26
 </t>
         </is>
       </c>
@@ -4718,7 +4718,7 @@
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">859
+          <t xml:space="preserve">253
 </t>
         </is>
       </c>
@@ -4736,13 +4736,13 @@
       </c>
       <c r="T29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8210
+          <t xml:space="preserve">8270
 </t>
         </is>
       </c>
       <c r="U29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">142
+          <t xml:space="preserve">942
 </t>
         </is>
       </c>
@@ -4760,7 +4760,7 @@
       </c>
       <c r="X29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2166
+          <t xml:space="preserve">2146
 </t>
         </is>
       </c>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11452
+          <t xml:space="preserve">1452
 </t>
         </is>
       </c>
@@ -4811,7 +4811,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11242
+          <t xml:space="preserve">1242
 </t>
         </is>
       </c>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1966
+          <t xml:space="preserve">2966
 </t>
         </is>
       </c>
@@ -4841,7 +4841,7 @@
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">288
+          <t xml:space="preserve">3288
 </t>
         </is>
       </c>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="N30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1259
+          <t xml:space="preserve">1239
 </t>
         </is>
       </c>
@@ -4883,13 +4883,13 @@
       </c>
       <c r="R30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1201
+          <t xml:space="preserve">1207
 </t>
         </is>
       </c>
       <c r="S30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1409
+          <t xml:space="preserve">12409
 </t>
         </is>
       </c>
@@ -4899,27 +4899,24 @@
 </t>
         </is>
       </c>
-      <c r="U30" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">180
-</t>
-        </is>
+      <c r="U30" s="3" t="n">
+        <v/>
       </c>
       <c r="V30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11261
+          <t xml:space="preserve">1261
 </t>
         </is>
       </c>
       <c r="W30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1158
+          <t xml:space="preserve">1159
 </t>
         </is>
       </c>
       <c r="X30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1329
+          <t xml:space="preserve">1359
 </t>
         </is>
       </c>
@@ -4931,7 +4928,7 @@
       </c>
       <c r="Z30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">281
+          <t xml:space="preserve">858
 </t>
         </is>
       </c>
@@ -4958,18 +4955,18 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>82</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9086
+          <t xml:space="preserve">906
 </t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2148
+          <t xml:space="preserve">248
 </t>
         </is>
       </c>
@@ -4999,7 +4996,7 @@
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 0
+          <t xml:space="preserve">9
 </t>
         </is>
       </c>
@@ -5023,7 +5020,7 @@
       </c>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">975
+          <t xml:space="preserve">9275
 </t>
         </is>
       </c>
@@ -5059,7 +5056,7 @@
       </c>
       <c r="U31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">188
+          <t xml:space="preserve">88
 </t>
         </is>
       </c>
@@ -5077,19 +5074,19 @@
       </c>
       <c r="X31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">972
+          <t xml:space="preserve">272
 </t>
         </is>
       </c>
       <c r="Y31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">249
+          <t xml:space="preserve">849
 </t>
         </is>
       </c>
       <c r="Z31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">42
+          <t xml:space="preserve">52
 </t>
         </is>
       </c>
@@ -5110,7 +5107,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">88169
+          <t xml:space="preserve">3847
 </t>
         </is>
       </c>
@@ -5122,13 +5119,13 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">193
+          <t xml:space="preserve">293
 </t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">252
+          <t xml:space="preserve">232
 </t>
         </is>
       </c>
@@ -5146,7 +5143,7 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">29
+          <t xml:space="preserve">23
 </t>
         </is>
       </c>
@@ -5176,7 +5173,7 @@
       </c>
       <c r="N32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">239
+          <t xml:space="preserve">235
 </t>
         </is>
       </c>
@@ -5206,7 +5203,7 @@
       </c>
       <c r="S32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2725
+          <t xml:space="preserve">275
 </t>
         </is>
       </c>
@@ -5218,31 +5215,30 @@
       </c>
       <c r="U32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">145
+          <t xml:space="preserve">175
 </t>
         </is>
       </c>
       <c r="V32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">274
-</t>
+          <t>93</t>
         </is>
       </c>
       <c r="W32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">238
+          <t xml:space="preserve">838
 </t>
         </is>
       </c>
       <c r="X32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">972
+          <t xml:space="preserve">272
 </t>
         </is>
       </c>
       <c r="Y32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">761
+          <t xml:space="preserve">76416
 </t>
         </is>
       </c>
@@ -5323,7 +5319,7 @@
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">815
+          <t xml:space="preserve">215
 </t>
         </is>
       </c>
@@ -5335,7 +5331,7 @@
       </c>
       <c r="N33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">178
+          <t xml:space="preserve">239
 </t>
         </is>
       </c>
@@ -5353,13 +5349,13 @@
       </c>
       <c r="Q33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">229
+          <t xml:space="preserve">289
 </t>
         </is>
       </c>
       <c r="R33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">206
+          <t xml:space="preserve">286
 </t>
         </is>
       </c>
@@ -5371,7 +5367,7 @@
       </c>
       <c r="T33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">209
+          <t xml:space="preserve">709
 </t>
         </is>
       </c>
@@ -5389,7 +5385,7 @@
       </c>
       <c r="W33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1238
+          <t xml:space="preserve">238
 </t>
         </is>
       </c>
@@ -5401,13 +5397,12 @@
       </c>
       <c r="Y33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">862
-</t>
+          <t>261</t>
         </is>
       </c>
       <c r="Z33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">125
+          <t xml:space="preserve">1445
 </t>
         </is>
       </c>
@@ -5446,13 +5441,13 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1267
+          <t xml:space="preserve">267
 </t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">104
+          <t xml:space="preserve">105
 </t>
         </is>
       </c>
@@ -5470,7 +5465,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">395
+          <t xml:space="preserve">95
 </t>
         </is>
       </c>
@@ -5512,13 +5507,13 @@
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">30
+          <t xml:space="preserve">305
 </t>
         </is>
       </c>
       <c r="R34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">238
+          <t xml:space="preserve">258
 </t>
         </is>
       </c>
@@ -5560,7 +5555,7 @@
       </c>
       <c r="Y34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1828
+          <t xml:space="preserve">828
 </t>
         </is>
       </c>
@@ -5593,118 +5588,117 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">2311
+</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>308</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">259
+</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">103
+</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">197
+</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24
+</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40
+</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">00
+</t>
+        </is>
+      </c>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">216
+</t>
+        </is>
+      </c>
+      <c r="M35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">213
+</t>
+        </is>
+      </c>
+      <c r="N35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">251
+</t>
+        </is>
+      </c>
+      <c r="O35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">972
+</t>
+        </is>
+      </c>
+      <c r="P35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">07
+</t>
+        </is>
+      </c>
+      <c r="Q35" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">311
 </t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">208
-</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1259
-</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">103
-</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">197
-</t>
-        </is>
-      </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">24
-</t>
-        </is>
-      </c>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40
-</t>
-        </is>
-      </c>
-      <c r="K35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">00
-</t>
-        </is>
-      </c>
-      <c r="L35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">216
-</t>
-        </is>
-      </c>
-      <c r="M35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">213
-</t>
-        </is>
-      </c>
-      <c r="N35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">251
-</t>
-        </is>
-      </c>
-      <c r="O35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">972
-</t>
-        </is>
-      </c>
-      <c r="P35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">071
-</t>
-        </is>
-      </c>
-      <c r="Q35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">311
-</t>
-        </is>
-      </c>
       <c r="R35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">249
+          <t xml:space="preserve">2469
 </t>
         </is>
       </c>
       <c r="S35" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">218
+</t>
+        </is>
+      </c>
+      <c r="T35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">613
+</t>
+        </is>
+      </c>
+      <c r="U35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">174
+</t>
+        </is>
+      </c>
+      <c r="V35" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">278
 </t>
         </is>
       </c>
-      <c r="T35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">613
-</t>
-        </is>
-      </c>
-      <c r="U35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">174
-</t>
-        </is>
-      </c>
-      <c r="V35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">218
-</t>
-        </is>
-      </c>
       <c r="W35" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">2166
@@ -5719,13 +5713,12 @@
       </c>
       <c r="Y35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">779
-</t>
+          <t>32</t>
         </is>
       </c>
       <c r="Z35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8111
+          <t xml:space="preserve">84
 </t>
         </is>
       </c>
@@ -5818,7 +5811,7 @@
       </c>
       <c r="O36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">985
+          <t xml:space="preserve">975
 </t>
         </is>
       </c>
@@ -5866,25 +5859,25 @@
       </c>
       <c r="W36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">246
+          <t xml:space="preserve">2466
 </t>
         </is>
       </c>
       <c r="X36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2839
+          <t xml:space="preserve">288
 </t>
         </is>
       </c>
       <c r="Y36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1720
+          <t xml:space="preserve">720
 </t>
         </is>
       </c>
       <c r="Z36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">110
+          <t xml:space="preserve">14110
 </t>
         </is>
       </c>
@@ -5965,13 +5958,13 @@
       </c>
       <c r="M37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1052
+          <t xml:space="preserve">1032
 </t>
         </is>
       </c>
       <c r="N37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1261
+          <t xml:space="preserve">1241
 </t>
         </is>
       </c>
@@ -5989,7 +5982,7 @@
       </c>
       <c r="Q37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1531
+          <t xml:space="preserve">1537
 </t>
         </is>
       </c>
@@ -6007,19 +6000,19 @@
       </c>
       <c r="T37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">82168
+          <t xml:space="preserve">3248
 </t>
         </is>
       </c>
       <c r="U37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">117
+          <t xml:space="preserve">197
 </t>
         </is>
       </c>
       <c r="V37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1268
+          <t xml:space="preserve">1368
 </t>
         </is>
       </c>
@@ -6031,19 +6024,19 @@
       </c>
       <c r="X37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1024
+          <t xml:space="preserve">1224
 </t>
         </is>
       </c>
       <c r="Y37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3982
+          <t xml:space="preserve">39282
 </t>
         </is>
       </c>
       <c r="Z37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8921
+          <t xml:space="preserve">397
 </t>
         </is>
       </c>
@@ -6094,7 +6087,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">198
+          <t xml:space="preserve">193
 </t>
         </is>
       </c>
@@ -6151,7 +6144,7 @@
       </c>
       <c r="R38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8252
+          <t xml:space="preserve">252
 </t>
         </is>
       </c>
@@ -6163,19 +6156,19 @@
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">620
+          <t xml:space="preserve">690
 </t>
         </is>
       </c>
       <c r="U38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">125
+          <t xml:space="preserve">155
 </t>
         </is>
       </c>
       <c r="V38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">874
+          <t xml:space="preserve">274
 </t>
         </is>
       </c>
@@ -6199,7 +6192,7 @@
       </c>
       <c r="Z38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5661
+          <t xml:space="preserve">79
 </t>
         </is>
       </c>
@@ -6220,13 +6213,13 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">32325
+          <t xml:space="preserve">3325
 </t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">182181
+          <t xml:space="preserve">319
 </t>
         </is>
       </c>
@@ -6250,7 +6243,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">193
+          <t xml:space="preserve">1193
 </t>
         </is>
       </c>
@@ -6268,7 +6261,7 @@
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">15
+          <t xml:space="preserve">12
 </t>
         </is>
       </c>
@@ -6304,13 +6297,13 @@
       </c>
       <c r="Q39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">119
+          <t xml:space="preserve">919
 </t>
         </is>
       </c>
       <c r="R39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1260
+          <t xml:space="preserve">260
 </t>
         </is>
       </c>
@@ -6328,19 +6321,19 @@
       </c>
       <c r="U39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">119
+          <t xml:space="preserve">113
 </t>
         </is>
       </c>
       <c r="V39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2491
+          <t xml:space="preserve">249
 </t>
         </is>
       </c>
       <c r="W39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">222
+          <t xml:space="preserve">232
 </t>
         </is>
       </c>
@@ -6358,7 +6351,7 @@
       </c>
       <c r="Z39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">86
+          <t xml:space="preserve">826
 </t>
         </is>
       </c>
@@ -6379,13 +6372,13 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">15341
+          <t xml:space="preserve">1537
 </t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">929
+          <t xml:space="preserve">229
 </t>
         </is>
       </c>
@@ -6415,13 +6408,13 @@
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">21
+          <t xml:space="preserve">27
 </t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">40
+          <t xml:space="preserve">50
 </t>
         </is>
       </c>
@@ -6481,7 +6474,7 @@
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">392
+          <t xml:space="preserve">592
 </t>
         </is>
       </c>
@@ -6499,19 +6492,19 @@
       </c>
       <c r="W40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1238
+          <t xml:space="preserve">238
 </t>
         </is>
       </c>
       <c r="X40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">269
+          <t xml:space="preserve">2869
 </t>
         </is>
       </c>
       <c r="Y40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">228
+          <t xml:space="preserve">720
 </t>
         </is>
       </c>
@@ -6538,7 +6531,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9656
+          <t xml:space="preserve">89856
 </t>
         </is>
       </c>
@@ -6609,73 +6602,73 @@
       </c>
       <c r="O41" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">990
+</t>
+        </is>
+      </c>
+      <c r="P41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02
+</t>
+        </is>
+      </c>
+      <c r="Q41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">223
+</t>
+        </is>
+      </c>
+      <c r="R41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">214
+</t>
+        </is>
+      </c>
+      <c r="S41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2169
+</t>
+        </is>
+      </c>
+      <c r="T41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">923
+</t>
+        </is>
+      </c>
+      <c r="U41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20
+</t>
+        </is>
+      </c>
+      <c r="V41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">226
+</t>
+        </is>
+      </c>
+      <c r="W41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">234
+</t>
+        </is>
+      </c>
+      <c r="X41" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">980
 </t>
         </is>
       </c>
-      <c r="P41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">02
-</t>
-        </is>
-      </c>
-      <c r="Q41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">223
-</t>
-        </is>
-      </c>
-      <c r="R41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">214
-</t>
-        </is>
-      </c>
-      <c r="S41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">249
-</t>
-        </is>
-      </c>
-      <c r="T41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">929
-</t>
-        </is>
-      </c>
-      <c r="U41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">28
-</t>
-        </is>
-      </c>
-      <c r="V41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2466
-</t>
-        </is>
-      </c>
-      <c r="W41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">234
-</t>
-        </is>
-      </c>
-      <c r="X41" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">292180
-</t>
-        </is>
-      </c>
       <c r="Y41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">905
+          <t xml:space="preserve">904
 </t>
         </is>
       </c>
       <c r="Z41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">189
+          <t xml:space="preserve">89
 </t>
         </is>
       </c>
@@ -6708,7 +6701,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8039
+          <t xml:space="preserve">203
 </t>
         </is>
       </c>
@@ -6720,7 +6713,7 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1113
+          <t xml:space="preserve">113
 </t>
         </is>
       </c>
@@ -6738,13 +6731,13 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">18
+          <t xml:space="preserve">1080
 </t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8281
+          <t xml:space="preserve">284
 </t>
         </is>
       </c>
@@ -6762,13 +6755,13 @@
       </c>
       <c r="N42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">262
+          <t xml:space="preserve">260
 </t>
         </is>
       </c>
       <c r="O42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">18990
+          <t xml:space="preserve">890
 </t>
         </is>
       </c>
@@ -6810,19 +6803,19 @@
       </c>
       <c r="V42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">28229
+          <t xml:space="preserve">227
 </t>
         </is>
       </c>
       <c r="W42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1825
+          <t xml:space="preserve">225
 </t>
         </is>
       </c>
       <c r="X42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1882
+          <t xml:space="preserve">28282
 </t>
         </is>
       </c>
@@ -6873,127 +6866,127 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">247
+</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">87
+</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">198
+</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20
+</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">37
+</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">00
+</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">216
+</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">215
+</t>
+        </is>
+      </c>
+      <c r="N43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">256
+</t>
+        </is>
+      </c>
+      <c r="O43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">990
+</t>
+        </is>
+      </c>
+      <c r="P43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02
+</t>
+        </is>
+      </c>
+      <c r="Q43" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">291
 </t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">87
-</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">198
-</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20
-</t>
-        </is>
-      </c>
-      <c r="J43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">137
-</t>
-        </is>
-      </c>
-      <c r="K43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">00
-</t>
-        </is>
-      </c>
-      <c r="L43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">216
-</t>
-        </is>
-      </c>
-      <c r="M43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">215
-</t>
-        </is>
-      </c>
-      <c r="N43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">256
-</t>
-        </is>
-      </c>
-      <c r="O43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">990
-</t>
-        </is>
-      </c>
-      <c r="P43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">02
-</t>
-        </is>
-      </c>
-      <c r="Q43" s="3" t="inlineStr">
+      <c r="R43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">255
+</t>
+        </is>
+      </c>
+      <c r="S43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">804
+</t>
+        </is>
+      </c>
+      <c r="T43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">756
+</t>
+        </is>
+      </c>
+      <c r="U43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">98
+</t>
+        </is>
+      </c>
+      <c r="V43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">218
+</t>
+        </is>
+      </c>
+      <c r="W43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">247
+</t>
+        </is>
+      </c>
+      <c r="X43" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">291
 </t>
         </is>
       </c>
-      <c r="R43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">256
-</t>
-        </is>
-      </c>
-      <c r="S43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">804
-</t>
-        </is>
-      </c>
-      <c r="T43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">756
-</t>
-        </is>
-      </c>
-      <c r="U43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">98
-</t>
-        </is>
-      </c>
-      <c r="V43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">218
-</t>
-        </is>
-      </c>
-      <c r="W43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2414
-</t>
-        </is>
-      </c>
-      <c r="X43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">291
-</t>
-        </is>
-      </c>
       <c r="Y43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">180
+          <t xml:space="preserve">780
 </t>
         </is>
       </c>
       <c r="Z43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1982
+          <t xml:space="preserve">82
 </t>
         </is>
       </c>
@@ -7014,13 +7007,13 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">659
+          <t xml:space="preserve">3659
 </t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">226
+          <t xml:space="preserve">226 1
 </t>
         </is>
       </c>
@@ -7044,7 +7037,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">894
+          <t xml:space="preserve">1194
 </t>
         </is>
       </c>
@@ -7068,13 +7061,13 @@
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">223
+          <t xml:space="preserve">2823
 </t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">223
+          <t xml:space="preserve">823
 </t>
         </is>
       </c>
@@ -7092,7 +7085,7 @@
       </c>
       <c r="P44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">80
+          <t xml:space="preserve">00
 </t>
         </is>
       </c>
@@ -7104,31 +7097,31 @@
       </c>
       <c r="R44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8264
+          <t xml:space="preserve">264
 </t>
         </is>
       </c>
       <c r="S44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">806
+          <t xml:space="preserve">304
 </t>
         </is>
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1620
+          <t xml:space="preserve">620
 </t>
         </is>
       </c>
       <c r="U44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">086
+          <t xml:space="preserve">186
 </t>
         </is>
       </c>
       <c r="V44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">285
+          <t xml:space="preserve">283
 </t>
         </is>
       </c>
@@ -7140,7 +7133,7 @@
       </c>
       <c r="X44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">828
+          <t xml:space="preserve">8282
 </t>
         </is>
       </c>
@@ -7179,37 +7172,37 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">191656
+          <t xml:space="preserve">19016
 </t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11280
+          <t xml:space="preserve">112986
 </t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">20261
+          <t xml:space="preserve">2261
 </t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">091
+          <t xml:space="preserve">021
 </t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11142
+          <t xml:space="preserve">111 42
 </t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11010
+          <t xml:space="preserve">0110
 </t>
         </is>
       </c>
@@ -7221,18 +7214,18 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>7431</t>
+          <t>7836</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">116659
+          <t xml:space="preserve">11665
 </t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1289
+          <t xml:space="preserve">1239
 </t>
         </is>
       </c>
@@ -7244,13 +7237,13 @@
       </c>
       <c r="O45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2928
+          <t xml:space="preserve">2938
 </t>
         </is>
       </c>
       <c r="P45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12
+          <t xml:space="preserve">13
 </t>
         </is>
       </c>
@@ -7262,25 +7255,25 @@
       </c>
       <c r="R45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">014691
+          <t xml:space="preserve">1491
 </t>
         </is>
       </c>
       <c r="S45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1741
+          <t xml:space="preserve">1211
 </t>
         </is>
       </c>
       <c r="T45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">14508
+          <t xml:space="preserve">12300
 </t>
         </is>
       </c>
       <c r="U45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">656
+          <t xml:space="preserve">686
 </t>
         </is>
       </c>
@@ -7292,24 +7285,24 @@
       </c>
       <c r="W45" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">1282
+</t>
+        </is>
+      </c>
+      <c r="X45" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">1722
 </t>
         </is>
       </c>
-      <c r="X45" s="3" t="inlineStr">
-        <is>
-          <t>845</t>
-        </is>
-      </c>
       <c r="Y45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9001
-</t>
+          <t>5034</t>
         </is>
       </c>
       <c r="Z45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">560
+          <t xml:space="preserve">160
 </t>
         </is>
       </c>
@@ -7354,7 +7347,7 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1215
+          <t xml:space="preserve">215
 </t>
         </is>
       </c>
@@ -7376,15 +7369,12 @@
 </t>
         </is>
       </c>
-      <c r="K46" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10
-</t>
-        </is>
+      <c r="K46" s="3" t="n">
+        <v/>
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2111
+          <t xml:space="preserve">211
 </t>
         </is>
       </c>
@@ -7402,7 +7392,7 @@
       </c>
       <c r="O46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">990
+          <t xml:space="preserve">1990
 </t>
         </is>
       </c>
@@ -7432,7 +7422,7 @@
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">729
+          <t xml:space="preserve">229
 </t>
         </is>
       </c>
@@ -7462,13 +7452,13 @@
       </c>
       <c r="Y46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">838
+          <t xml:space="preserve">888
 </t>
         </is>
       </c>
       <c r="Z46" s="3" t="inlineStr">
         <is>
-          <t>625</t>
+          <t>62</t>
         </is>
       </c>
       <c r="AA46" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Updates to the initial v1.0 modules. Here we also add QA/QC checks for precipitation, dry and wet bulb temperatures, vapour pressure and relative humidity
</commit_message>
<xml_diff>
--- a/results/01_pre_QA_QC_transcribed_hydroclimate_data/203/203_196905_SF.JPG_pre_QA_QC.xlsx
+++ b/results/01_pre_QA_QC_transcribed_hydroclimate_data/203/203_196905_SF.JPG_pre_QA_QC.xlsx
@@ -679,13 +679,13 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1862
+          <t xml:space="preserve">136
 </t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">281
+          <t xml:space="preserve">288
 </t>
         </is>
       </c>
@@ -703,19 +703,19 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">872
+          <t xml:space="preserve">87
 </t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">182
+          <t xml:space="preserve">1882
 </t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">118
+          <t xml:space="preserve">17
 </t>
         </is>
       </c>
@@ -727,7 +727,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">00
+          <t xml:space="preserve">80
 </t>
         </is>
       </c>
@@ -805,7 +805,7 @@
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">262
+          <t xml:space="preserve">1262
 </t>
         </is>
       </c>
@@ -838,7 +838,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4038
+          <t xml:space="preserve">2403
 </t>
         </is>
       </c>
@@ -868,7 +868,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">168
+          <t xml:space="preserve">14168
 </t>
         </is>
       </c>
@@ -970,7 +970,7 @@
       </c>
       <c r="Y5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">71740
+          <t xml:space="preserve">770
 </t>
         </is>
       </c>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">288
+          <t xml:space="preserve">188
 </t>
         </is>
       </c>
@@ -1027,13 +1027,13 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1152
+          <t xml:space="preserve">172
 </t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">146
+          <t xml:space="preserve">46
 </t>
         </is>
       </c>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">928
+          <t xml:space="preserve">1558
 </t>
         </is>
       </c>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="V6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">281
+          <t xml:space="preserve">287
 </t>
         </is>
       </c>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">348
+          <t xml:space="preserve">34
 </t>
         </is>
       </c>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2720
+          <t xml:space="preserve">220
 </t>
         </is>
       </c>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">847
+          <t xml:space="preserve">647
 </t>
         </is>
       </c>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">235
+          <t xml:space="preserve">23
 </t>
         </is>
       </c>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">80
+          <t xml:space="preserve">00
 </t>
         </is>
       </c>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="R7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">22
+          <t xml:space="preserve">25
 </t>
         </is>
       </c>
@@ -1258,19 +1258,19 @@
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">206
+          <t xml:space="preserve">506
 </t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">265
+          <t xml:space="preserve">26
 </t>
         </is>
       </c>
       <c r="V7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">295
+          <t xml:space="preserve">29
 </t>
         </is>
       </c>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="X7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">273
+          <t xml:space="preserve">27
 </t>
         </is>
       </c>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1120
+          <t xml:space="preserve">1190
 </t>
         </is>
       </c>
@@ -1357,13 +1357,13 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">140
+          <t xml:space="preserve">40
 </t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">309
+          <t xml:space="preserve">2309
 </t>
         </is>
       </c>
@@ -1387,7 +1387,7 @@
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2965
+          <t xml:space="preserve">965
 </t>
         </is>
       </c>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="Z8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">206
+          <t xml:space="preserve">06
 </t>
         </is>
       </c>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">17832
+          <t xml:space="preserve">1783
 </t>
         </is>
       </c>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">230 8
+          <t xml:space="preserve">1308
 </t>
         </is>
       </c>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">168
+          <t xml:space="preserve">165
 </t>
         </is>
       </c>
@@ -1522,8 +1522,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">309
-</t>
+          <t>308</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
@@ -1540,19 +1539,19 @@
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1128
+          <t xml:space="preserve">1188
 </t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4942
+          <t xml:space="preserve">4945
 </t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">112
+          <t xml:space="preserve">12
 </t>
         </is>
       </c>
@@ -1576,13 +1575,13 @@
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3299
+          <t xml:space="preserve">23299
 </t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">820
+          <t xml:space="preserve">810
 </t>
         </is>
       </c>
@@ -1606,7 +1605,7 @@
       </c>
       <c r="Y9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">37888
+          <t xml:space="preserve">3888
 </t>
         </is>
       </c>
@@ -1633,7 +1632,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">354
+          <t xml:space="preserve">3567
 </t>
         </is>
       </c>
@@ -1645,7 +1644,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">198
+          <t xml:space="preserve">194
 </t>
         </is>
       </c>
@@ -1679,11 +1678,8 @@
 </t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11 1
-</t>
-        </is>
+      <c r="K10" s="3" t="n">
+        <v/>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
@@ -1717,7 +1713,7 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1299
+          <t xml:space="preserve">299
 </t>
         </is>
       </c>
@@ -1765,7 +1761,7 @@
       </c>
       <c r="Y10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">728
+          <t xml:space="preserve">778
 </t>
         </is>
       </c>
@@ -1828,52 +1824,52 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">116
+</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28
+</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">00
+</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">212
+</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">209
+</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">245
+</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">973
+</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">06
 </t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">28
-</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">00
-</t>
-        </is>
-      </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">212
-</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">209
-</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">245
-</t>
-        </is>
-      </c>
-      <c r="O11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">213
-</t>
-        </is>
-      </c>
-      <c r="P11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">06
-</t>
-        </is>
-      </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">299
@@ -1882,7 +1878,7 @@
       </c>
       <c r="R11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">235
+          <t xml:space="preserve">255
 </t>
         </is>
       </c>
@@ -1912,7 +1908,7 @@
       </c>
       <c r="W11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">949
+          <t xml:space="preserve">249
 </t>
         </is>
       </c>
@@ -1924,13 +1920,13 @@
       </c>
       <c r="Y11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8940
+          <t xml:space="preserve">840
 </t>
         </is>
       </c>
       <c r="Z11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">58
+          <t xml:space="preserve">1598
 </t>
         </is>
       </c>
@@ -1951,19 +1947,19 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2421
+          <t xml:space="preserve">3471
 </t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">818
+          <t xml:space="preserve">318
 </t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">826
+          <t xml:space="preserve">226
 </t>
         </is>
       </c>
@@ -1993,7 +1989,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">146
+          <t xml:space="preserve">46
 </t>
         </is>
       </c>
@@ -2023,7 +2019,7 @@
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9275
+          <t xml:space="preserve">275
 </t>
         </is>
       </c>
@@ -2053,7 +2049,7 @@
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">598
+          <t xml:space="preserve">588
 </t>
         </is>
       </c>
@@ -2065,7 +2061,7 @@
       </c>
       <c r="V12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">219
+          <t xml:space="preserve">279
 </t>
         </is>
       </c>
@@ -2089,7 +2085,7 @@
       </c>
       <c r="Z12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">817
+          <t xml:space="preserve">87
 </t>
         </is>
       </c>
@@ -2122,7 +2118,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">204
+          <t xml:space="preserve">201
 </t>
         </is>
       </c>
@@ -2152,7 +2148,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">160
+          <t xml:space="preserve">60
 </t>
         </is>
       </c>
@@ -2230,7 +2226,7 @@
       </c>
       <c r="W13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">248
+          <t xml:space="preserve">24
 </t>
         </is>
       </c>
@@ -2248,7 +2244,7 @@
       </c>
       <c r="Z13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">185
+          <t xml:space="preserve">25
 </t>
         </is>
       </c>
@@ -2275,7 +2271,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3071
+          <t xml:space="preserve">307
 </t>
         </is>
       </c>
@@ -2305,13 +2301,13 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">115
+          <t xml:space="preserve">15
 </t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">821
+          <t xml:space="preserve">21
 </t>
         </is>
       </c>
@@ -2353,7 +2349,7 @@
       </c>
       <c r="Q14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">824
+          <t xml:space="preserve">224
 </t>
         </is>
       </c>
@@ -2365,8 +2361,7 @@
       </c>
       <c r="S14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">242
-</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="T14" s="3" t="inlineStr">
@@ -2405,8 +2400,11 @@
 </t>
         </is>
       </c>
-      <c r="Z14" s="3" t="n">
-        <v/>
+      <c r="Z14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">09
+</t>
+        </is>
       </c>
       <c r="AA14" s="3" t="inlineStr">
         <is>
@@ -2473,31 +2471,31 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">237
+          <t xml:space="preserve">257
 </t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">286
+</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">216
 </t>
         </is>
       </c>
-      <c r="M15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">216
-</t>
-        </is>
-      </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">258
+          <t xml:space="preserve">298
 </t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1002
+          <t xml:space="preserve">1000
 </t>
         </is>
       </c>
@@ -2584,30 +2582,31 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12212
+          <t xml:space="preserve">15912
 </t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1679
+          <t xml:space="preserve">1579
 </t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>12551</t>
+          <t xml:space="preserve">1055
+</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1319
+          <t xml:space="preserve">1317
 </t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">524
+          <t xml:space="preserve">3524
 </t>
         </is>
       </c>
@@ -2637,25 +2636,25 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1106
+          <t xml:space="preserve">11106
 </t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1098
+          <t xml:space="preserve">1095
 </t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12307
+          <t xml:space="preserve">1307
 </t>
         </is>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">14901
+          <t xml:space="preserve">24901
 </t>
         </is>
       </c>
@@ -2673,7 +2672,7 @@
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12219
+          <t xml:space="preserve">1219
 </t>
         </is>
       </c>
@@ -2703,7 +2702,7 @@
       </c>
       <c r="W16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1207
+          <t xml:space="preserve">21207
 </t>
         </is>
       </c>
@@ -2715,14 +2714,13 @@
       </c>
       <c r="Y16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">14076
+          <t xml:space="preserve">4074
 </t>
         </is>
       </c>
       <c r="Z16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">344
-</t>
+          <t>344</t>
         </is>
       </c>
       <c r="AA16" s="3" t="inlineStr">
@@ -2748,7 +2746,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">316
+          <t xml:space="preserve">2316
 </t>
         </is>
       </c>
@@ -2790,7 +2788,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0060
+          <t xml:space="preserve">1
 </t>
         </is>
       </c>
@@ -2814,13 +2812,13 @@
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9280
+          <t xml:space="preserve">2980
 </t>
         </is>
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">04
+          <t xml:space="preserve">14
 </t>
         </is>
       </c>
@@ -2844,7 +2842,7 @@
       </c>
       <c r="T17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">664
+          <t xml:space="preserve">1664
 </t>
         </is>
       </c>
@@ -2856,12 +2854,13 @@
       </c>
       <c r="V17" s="3" t="inlineStr">
         <is>
-          <t>83</t>
+          <t xml:space="preserve">267
+</t>
         </is>
       </c>
       <c r="W17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">241
+          <t xml:space="preserve">2241
 </t>
         </is>
       </c>
@@ -2879,7 +2878,7 @@
       </c>
       <c r="Z17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">169
+          <t xml:space="preserve">69
 </t>
         </is>
       </c>
@@ -2918,16 +2917,19 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">261
-</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="n">
-        <v/>
+          <t xml:space="preserve">267
+</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">109
+</t>
+        </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">804
+          <t xml:space="preserve">204
 </t>
         </is>
       </c>
@@ -2939,20 +2941,18 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">143
+          <t xml:space="preserve">43
 </t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">104
-</t>
+          <t>40</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">214
-</t>
+          <t>244</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">973
+          <t xml:space="preserve">1973
 </t>
         </is>
       </c>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="Q18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">321
+          <t xml:space="preserve">2321
 </t>
         </is>
       </c>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">380
+          <t xml:space="preserve">580
 </t>
         </is>
       </c>
@@ -3017,19 +3017,18 @@
       </c>
       <c r="W18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">244
-</t>
+          <t>244</t>
         </is>
       </c>
       <c r="X18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">219
+          <t xml:space="preserve">279
 </t>
         </is>
       </c>
       <c r="Y18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">719
+          <t xml:space="preserve">1717
 </t>
         </is>
       </c>
@@ -3086,7 +3085,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2914
+          <t xml:space="preserve">214
 </t>
         </is>
       </c>
@@ -3134,7 +3133,7 @@
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">106
+          <t xml:space="preserve">06
 </t>
         </is>
       </c>
@@ -3176,7 +3175,7 @@
       </c>
       <c r="W19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1289
+          <t xml:space="preserve">229
 </t>
         </is>
       </c>
@@ -3194,7 +3193,7 @@
       </c>
       <c r="Z19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">83
+          <t xml:space="preserve">123
 </t>
         </is>
       </c>
@@ -3221,25 +3220,25 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">314
+          <t xml:space="preserve">1314
 </t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2185
+          <t xml:space="preserve">215
 </t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">285
+          <t xml:space="preserve">1265
 </t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">199
+          <t xml:space="preserve">299
 </t>
         </is>
       </c>
@@ -3257,7 +3256,7 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">145
+          <t xml:space="preserve">45
 </t>
         </is>
       </c>
@@ -3281,7 +3280,7 @@
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">254
+          <t xml:space="preserve">251
 </t>
         </is>
       </c>
@@ -3293,7 +3292,7 @@
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">04
+          <t xml:space="preserve">104
 </t>
         </is>
       </c>
@@ -3311,13 +3310,13 @@
       </c>
       <c r="S20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2175
+          <t xml:space="preserve">275
 </t>
         </is>
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">123
+          <t xml:space="preserve">623
 </t>
         </is>
       </c>
@@ -3329,13 +3328,13 @@
       </c>
       <c r="V20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">273
+          <t xml:space="preserve">27
 </t>
         </is>
       </c>
       <c r="W20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">228
+          <t xml:space="preserve">238
 </t>
         </is>
       </c>
@@ -3347,13 +3346,13 @@
       </c>
       <c r="Y20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">7250
+          <t xml:space="preserve">850
 </t>
         </is>
       </c>
       <c r="Z20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">91
+          <t xml:space="preserve">191
 </t>
         </is>
       </c>
@@ -3380,7 +3379,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3072
+          <t xml:space="preserve">307
 </t>
         </is>
       </c>
@@ -3494,7 +3493,7 @@
       </c>
       <c r="W21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2266
+          <t xml:space="preserve">246
 </t>
         </is>
       </c>
@@ -3533,7 +3532,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3993
+          <t xml:space="preserve">23993
 </t>
         </is>
       </c>
@@ -3557,7 +3556,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">118
+          <t xml:space="preserve">11
 </t>
         </is>
       </c>
@@ -3581,7 +3580,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">27
+          <t xml:space="preserve">77
 </t>
         </is>
       </c>
@@ -3605,13 +3604,13 @@
       </c>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">975
+          <t xml:space="preserve">97
 </t>
         </is>
       </c>
       <c r="P22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">04
+          <t xml:space="preserve">014
 </t>
         </is>
       </c>
@@ -3623,7 +3622,7 @@
       </c>
       <c r="R22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">299
+          <t xml:space="preserve">259
 </t>
         </is>
       </c>
@@ -3647,7 +3646,7 @@
       </c>
       <c r="V22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8265
+          <t xml:space="preserve">265
 </t>
         </is>
       </c>
@@ -3671,7 +3670,7 @@
       </c>
       <c r="Z22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1449
+          <t xml:space="preserve">649
 </t>
         </is>
       </c>
@@ -3698,7 +3697,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1675
+          <t xml:space="preserve">1575
 </t>
         </is>
       </c>
@@ -3710,12 +3709,13 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>1388</t>
+          <t xml:space="preserve">1324
+</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">203
+          <t xml:space="preserve">503
 </t>
         </is>
       </c>
@@ -3733,12 +3733,14 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>104</t>
+          <t xml:space="preserve">193
+</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>491</t>
+          <t xml:space="preserve">193
+</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
@@ -3749,7 +3751,7 @@
       </c>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11070
+          <t xml:space="preserve">107
 </t>
         </is>
       </c>
@@ -3791,14 +3793,13 @@
       </c>
       <c r="T23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3251
+          <t xml:space="preserve">3257
 </t>
         </is>
       </c>
       <c r="U23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">794
-</t>
+          <t>724</t>
         </is>
       </c>
       <c r="V23" s="3" t="inlineStr">
@@ -3809,7 +3810,7 @@
       </c>
       <c r="W23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0203
+          <t xml:space="preserve">11203
 </t>
         </is>
       </c>
@@ -3827,7 +3828,8 @@
       </c>
       <c r="Z23" s="3" t="inlineStr">
         <is>
-          <t>3625</t>
+          <t xml:space="preserve">367
+</t>
         </is>
       </c>
       <c r="AA23" s="3" t="inlineStr">
@@ -3847,7 +3849,8 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>3432</t>
+          <t xml:space="preserve">3479
+</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -3864,7 +3867,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">263
+          <t xml:space="preserve">265
 </t>
         </is>
       </c>
@@ -3892,11 +3895,8 @@
 </t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1
-</t>
-        </is>
+      <c r="K24" s="3" t="n">
+        <v/>
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
@@ -3936,13 +3936,13 @@
       </c>
       <c r="R24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">856
+          <t xml:space="preserve">256
 </t>
         </is>
       </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">294
+          <t xml:space="preserve">894
 </t>
         </is>
       </c>
@@ -3972,18 +3972,19 @@
       </c>
       <c r="X24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">232
+          <t xml:space="preserve">222
 </t>
         </is>
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
-          <t>29813</t>
+          <t xml:space="preserve">798
+</t>
         </is>
       </c>
       <c r="Z24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">73
+          <t xml:space="preserve">173
 </t>
         </is>
       </c>
@@ -4022,7 +4023,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">235
+          <t xml:space="preserve">1235
 </t>
         </is>
       </c>
@@ -4064,8 +4065,7 @@
       </c>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">221
-</t>
+          <t>981</t>
         </is>
       </c>
       <c r="N25" s="3" t="inlineStr">
@@ -4112,13 +4112,13 @@
       </c>
       <c r="U25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">53
+          <t xml:space="preserve">93
 </t>
         </is>
       </c>
       <c r="V25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2144
+          <t xml:space="preserve">244
 </t>
         </is>
       </c>
@@ -4136,12 +4136,15 @@
       </c>
       <c r="Y25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">87817
-</t>
-        </is>
-      </c>
-      <c r="Z25" s="3" t="n">
-        <v/>
+          <t xml:space="preserve">877
+</t>
+        </is>
+      </c>
+      <c r="Z25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38
+</t>
+        </is>
       </c>
       <c r="AA25" s="3" t="inlineStr">
         <is>
@@ -4172,7 +4175,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">210
+          <t xml:space="preserve">200
 </t>
         </is>
       </c>
@@ -4208,7 +4211,7 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">61
+          <t xml:space="preserve">67
 </t>
         </is>
       </c>
@@ -4262,13 +4265,13 @@
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1920
+          <t xml:space="preserve">920
 </t>
         </is>
       </c>
       <c r="U26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">24
+          <t xml:space="preserve">28
 </t>
         </is>
       </c>
@@ -4292,13 +4295,13 @@
       </c>
       <c r="Y26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0918
+          <t xml:space="preserve">918
 </t>
         </is>
       </c>
       <c r="Z26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">24
+          <t xml:space="preserve">124
 </t>
         </is>
       </c>
@@ -4325,7 +4328,8 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>305</t>
+          <t xml:space="preserve">205
+</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -4336,12 +4340,13 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>255</t>
+          <t xml:space="preserve">255
+</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">199
+          <t xml:space="preserve">99
 </t>
         </is>
       </c>
@@ -4371,7 +4376,8 @@
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>504</t>
+          <t xml:space="preserve">207
+</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
@@ -4388,7 +4394,7 @@
       </c>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">980
+          <t xml:space="preserve">2980
 </t>
         </is>
       </c>
@@ -4418,7 +4424,7 @@
       </c>
       <c r="T27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">232
+          <t xml:space="preserve">732
 </t>
         </is>
       </c>
@@ -4430,7 +4436,7 @@
       </c>
       <c r="V27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">28269
+          <t xml:space="preserve">269
 </t>
         </is>
       </c>
@@ -4442,7 +4448,7 @@
       </c>
       <c r="X27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2890
+          <t xml:space="preserve">290
 </t>
         </is>
       </c>
@@ -4454,7 +4460,7 @@
       </c>
       <c r="Z27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">64
+          <t xml:space="preserve">164
 </t>
         </is>
       </c>
@@ -4481,7 +4487,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">318
+          <t xml:space="preserve">238
 </t>
         </is>
       </c>
@@ -4547,13 +4553,13 @@
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">97
+          <t xml:space="preserve">973
 </t>
         </is>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">18
+          <t xml:space="preserve">08
 </t>
         </is>
       </c>
@@ -4571,7 +4577,7 @@
       </c>
       <c r="S28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">272
+          <t xml:space="preserve">27
 </t>
         </is>
       </c>
@@ -4646,7 +4652,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">20805
+          <t xml:space="preserve">205
 </t>
         </is>
       </c>
@@ -4658,13 +4664,13 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1110
+          <t xml:space="preserve">110
 </t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">192
+          <t xml:space="preserve">1692
 </t>
         </is>
       </c>
@@ -4688,7 +4694,7 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">211
+          <t xml:space="preserve">201
 </t>
         </is>
       </c>
@@ -4706,7 +4712,7 @@
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">953
+          <t xml:space="preserve">25
 </t>
         </is>
       </c>
@@ -4718,7 +4724,7 @@
       </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">253
+          <t xml:space="preserve">825
 </t>
         </is>
       </c>
@@ -4736,13 +4742,13 @@
       </c>
       <c r="T29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8270
+          <t xml:space="preserve">270
 </t>
         </is>
       </c>
       <c r="U29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">942
+          <t xml:space="preserve">42
 </t>
         </is>
       </c>
@@ -4760,14 +4766,13 @@
       </c>
       <c r="X29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2146
+          <t xml:space="preserve">246
 </t>
         </is>
       </c>
       <c r="Y29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">908
-</t>
+          <t>9121</t>
         </is>
       </c>
       <c r="Z29" s="3" t="inlineStr">
@@ -4793,7 +4798,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">110562
+          <t xml:space="preserve">10562
 </t>
         </is>
       </c>
@@ -4835,13 +4840,13 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1110
+          <t xml:space="preserve">110
 </t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3288
+          <t xml:space="preserve">388
 </t>
         </is>
       </c>
@@ -4865,7 +4870,7 @@
       </c>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4876
+          <t xml:space="preserve">24876
 </t>
         </is>
       </c>
@@ -4889,7 +4894,7 @@
       </c>
       <c r="S30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12409
+          <t xml:space="preserve">1409
 </t>
         </is>
       </c>
@@ -4899,12 +4904,15 @@
 </t>
         </is>
       </c>
-      <c r="U30" s="3" t="n">
-        <v/>
+      <c r="U30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">195
+</t>
+        </is>
       </c>
       <c r="V30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1261
+          <t xml:space="preserve">11261
 </t>
         </is>
       </c>
@@ -4922,13 +4930,13 @@
       </c>
       <c r="Y30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">14247
+          <t xml:space="preserve">14287
 </t>
         </is>
       </c>
       <c r="Z30" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">858
+          <t xml:space="preserve">258
 </t>
         </is>
       </c>
@@ -4955,72 +4963,70 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>82</t>
+          <t xml:space="preserve">290
+</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">906
+          <t xml:space="preserve">206
 </t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">1248
+</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">84
+</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">193
+</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14
+</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22
+</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="n">
+        <v/>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">213
+</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">210
+</t>
+        </is>
+      </c>
+      <c r="N31" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">248
 </t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">84
-</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">193
-</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14
-</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22
-</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9
-</t>
-        </is>
-      </c>
-      <c r="L31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">213
-</t>
-        </is>
-      </c>
-      <c r="M31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">210
-</t>
-        </is>
-      </c>
-      <c r="N31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">248
-</t>
-        </is>
-      </c>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9275
+          <t xml:space="preserve">975
 </t>
         </is>
       </c>
@@ -5056,19 +5062,19 @@
       </c>
       <c r="U31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">88
+          <t xml:space="preserve">82
 </t>
         </is>
       </c>
       <c r="V31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">252
+          <t xml:space="preserve">1252
 </t>
         </is>
       </c>
       <c r="W31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">232
+          <t xml:space="preserve">1232
 </t>
         </is>
       </c>
@@ -5080,7 +5086,7 @@
       </c>
       <c r="Y31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">849
+          <t xml:space="preserve">249
 </t>
         </is>
       </c>
@@ -5119,13 +5125,13 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">293
+          <t xml:space="preserve">193
 </t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">232
+          <t xml:space="preserve">252
 </t>
         </is>
       </c>
@@ -5173,7 +5179,7 @@
       </c>
       <c r="N32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">235
+          <t xml:space="preserve">239
 </t>
         </is>
       </c>
@@ -5221,12 +5227,13 @@
       </c>
       <c r="V32" s="3" t="inlineStr">
         <is>
-          <t>93</t>
+          <t xml:space="preserve">274
+</t>
         </is>
       </c>
       <c r="W32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">838
+          <t xml:space="preserve">238
 </t>
         </is>
       </c>
@@ -5238,13 +5245,13 @@
       </c>
       <c r="Y32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">76416
+          <t xml:space="preserve">7466
 </t>
         </is>
       </c>
       <c r="Z32" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">193
+          <t xml:space="preserve">1953
 </t>
         </is>
       </c>
@@ -5271,7 +5278,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">292
+          <t xml:space="preserve">12292
 </t>
         </is>
       </c>
@@ -5301,7 +5308,7 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">10
+          <t xml:space="preserve">110
 </t>
         </is>
       </c>
@@ -5313,7 +5320,7 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">148
+          <t xml:space="preserve">48
 </t>
         </is>
       </c>
@@ -5331,7 +5338,7 @@
       </c>
       <c r="N33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">239
+          <t xml:space="preserve">254
 </t>
         </is>
       </c>
@@ -5355,7 +5362,7 @@
       </c>
       <c r="R33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">286
+          <t xml:space="preserve">216
 </t>
         </is>
       </c>
@@ -5397,12 +5404,12 @@
       </c>
       <c r="Y33" s="3" t="inlineStr">
         <is>
-          <t>261</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Z33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1445
+          <t xml:space="preserve">145
 </t>
         </is>
       </c>
@@ -5429,7 +5436,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2319
+          <t xml:space="preserve">319
 </t>
         </is>
       </c>
@@ -5465,7 +5472,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">95
+          <t xml:space="preserve">35
 </t>
         </is>
       </c>
@@ -5495,7 +5502,7 @@
       </c>
       <c r="O34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">990
+          <t xml:space="preserve">1990
 </t>
         </is>
       </c>
@@ -5513,7 +5520,7 @@
       </c>
       <c r="R34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">258
+          <t xml:space="preserve">2358
 </t>
         </is>
       </c>
@@ -5555,7 +5562,7 @@
       </c>
       <c r="Y34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">828
+          <t xml:space="preserve">820
 </t>
         </is>
       </c>
@@ -5582,7 +5589,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3534
+          <t xml:space="preserve">3531
 </t>
         </is>
       </c>
@@ -5594,7 +5601,8 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>308</t>
+          <t xml:space="preserve">208
+</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -5653,7 +5661,7 @@
       </c>
       <c r="O35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">972
+          <t xml:space="preserve">2972
 </t>
         </is>
       </c>
@@ -5677,7 +5685,7 @@
       </c>
       <c r="S35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">218
+          <t xml:space="preserve">278
 </t>
         </is>
       </c>
@@ -5713,7 +5721,8 @@
       </c>
       <c r="Y35" s="3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t xml:space="preserve">776
+</t>
         </is>
       </c>
       <c r="Z35" s="3" t="inlineStr">
@@ -5763,7 +5772,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1112
+          <t xml:space="preserve">112
 </t>
         </is>
       </c>
@@ -5811,8 +5820,7 @@
       </c>
       <c r="O36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">975
-</t>
+          <t>9251</t>
         </is>
       </c>
       <c r="P36" s="3" t="inlineStr">
@@ -5859,25 +5867,25 @@
       </c>
       <c r="W36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2466
+          <t xml:space="preserve">246
 </t>
         </is>
       </c>
       <c r="X36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">288
+          <t xml:space="preserve">283
 </t>
         </is>
       </c>
       <c r="Y36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">720
+          <t xml:space="preserve">1720
 </t>
         </is>
       </c>
       <c r="Z36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">14110
+          <t xml:space="preserve">1110
 </t>
         </is>
       </c>
@@ -5904,13 +5912,13 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1554
+          <t xml:space="preserve">141554
 </t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1020
+          <t xml:space="preserve">102 0
 </t>
         </is>
       </c>
@@ -5934,7 +5942,7 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1101
+          <t xml:space="preserve">11 01
 </t>
         </is>
       </c>
@@ -5958,7 +5966,7 @@
       </c>
       <c r="M37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1032
+          <t xml:space="preserve">1052
 </t>
         </is>
       </c>
@@ -5976,7 +5984,7 @@
       </c>
       <c r="P37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">17 1
+          <t xml:space="preserve">17
 </t>
         </is>
       </c>
@@ -5994,19 +6002,19 @@
       </c>
       <c r="S37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1431
+          <t xml:space="preserve">11431
 </t>
         </is>
       </c>
       <c r="T37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3248
+          <t xml:space="preserve">23248
 </t>
         </is>
       </c>
       <c r="U37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">197
+          <t xml:space="preserve">797
 </t>
         </is>
       </c>
@@ -6030,13 +6038,13 @@
       </c>
       <c r="Y37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">39282
+          <t xml:space="preserve">3922
 </t>
         </is>
       </c>
       <c r="Z37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">397
+          <t xml:space="preserve">1397
 </t>
         </is>
       </c>
@@ -6063,7 +6071,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">310
+          <t xml:space="preserve">319
 </t>
         </is>
       </c>
@@ -6126,7 +6134,7 @@
       </c>
       <c r="O38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">985
+          <t xml:space="preserve">98
 </t>
         </is>
       </c>
@@ -6156,7 +6164,7 @@
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">690
+          <t xml:space="preserve">650
 </t>
         </is>
       </c>
@@ -6168,7 +6176,7 @@
       </c>
       <c r="V38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">274
+          <t xml:space="preserve">874
 </t>
         </is>
       </c>
@@ -6180,13 +6188,13 @@
       </c>
       <c r="X38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">885
+          <t xml:space="preserve">285
 </t>
         </is>
       </c>
       <c r="Y38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">780
+          <t xml:space="preserve">291
 </t>
         </is>
       </c>
@@ -6237,13 +6245,13 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1217
+          <t xml:space="preserve">117
 </t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1193
+          <t xml:space="preserve">193
 </t>
         </is>
       </c>
@@ -6261,7 +6269,7 @@
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12
+          <t xml:space="preserve">6
 </t>
         </is>
       </c>
@@ -6297,7 +6305,7 @@
       </c>
       <c r="Q39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">919
+          <t xml:space="preserve">319
 </t>
         </is>
       </c>
@@ -6321,13 +6329,13 @@
       </c>
       <c r="U39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">113
+          <t xml:space="preserve">183
 </t>
         </is>
       </c>
       <c r="V39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">249
+          <t xml:space="preserve">247
 </t>
         </is>
       </c>
@@ -6339,7 +6347,7 @@
       </c>
       <c r="X39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">27
+          <t xml:space="preserve">275
 </t>
         </is>
       </c>
@@ -6351,7 +6359,7 @@
       </c>
       <c r="Z39" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">826
+          <t xml:space="preserve">236
 </t>
         </is>
       </c>
@@ -6372,13 +6380,13 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1537
+          <t xml:space="preserve">14537
 </t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">229
+          <t xml:space="preserve">329
 </t>
         </is>
       </c>
@@ -6498,7 +6506,7 @@
       </c>
       <c r="X40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2869
+          <t xml:space="preserve">269
 </t>
         </is>
       </c>
@@ -6510,7 +6518,7 @@
       </c>
       <c r="Z40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1016
+          <t xml:space="preserve">104
 </t>
         </is>
       </c>
@@ -6531,13 +6539,13 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">89856
+          <t xml:space="preserve">2656
 </t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">316
+          <t xml:space="preserve">2316
 </t>
         </is>
       </c>
@@ -6549,7 +6557,7 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8256
+          <t xml:space="preserve">256
 </t>
         </is>
       </c>
@@ -6579,7 +6587,7 @@
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>44</t>
         </is>
       </c>
       <c r="L41" s="3" t="inlineStr">
@@ -6626,7 +6634,7 @@
       </c>
       <c r="S41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2169
+          <t xml:space="preserve">249
 </t>
         </is>
       </c>
@@ -6644,7 +6652,7 @@
       </c>
       <c r="V41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">226
+          <t xml:space="preserve">2116
 </t>
         </is>
       </c>
@@ -6656,19 +6664,19 @@
       </c>
       <c r="X41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">980
+          <t xml:space="preserve">280
 </t>
         </is>
       </c>
       <c r="Y41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">904
+          <t xml:space="preserve">1905
 </t>
         </is>
       </c>
       <c r="Z41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">89
+          <t xml:space="preserve">29
 </t>
         </is>
       </c>
@@ -6689,7 +6697,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8363
+          <t xml:space="preserve">2363
 </t>
         </is>
       </c>
@@ -6731,13 +6739,13 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1080
+          <t xml:space="preserve">12
 </t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">284
+          <t xml:space="preserve">287
 </t>
         </is>
       </c>
@@ -6791,31 +6799,31 @@
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">977
+          <t xml:space="preserve">972
 </t>
         </is>
       </c>
       <c r="U42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">08
+          <t xml:space="preserve">07
 </t>
         </is>
       </c>
       <c r="V42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">227
+          <t xml:space="preserve">247
 </t>
         </is>
       </c>
       <c r="W42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">225
+          <t xml:space="preserve">235
 </t>
         </is>
       </c>
       <c r="X42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">28282
+          <t xml:space="preserve">282
 </t>
         </is>
       </c>
@@ -6825,11 +6833,8 @@
 </t>
         </is>
       </c>
-      <c r="Z42" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">29
-</t>
-        </is>
+      <c r="Z42" s="3" t="n">
+        <v/>
       </c>
       <c r="AA42" s="3" t="inlineStr">
         <is>
@@ -6866,116 +6871,115 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">257
+</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">87
+</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">198
+</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20
+</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">37
+</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">00
+</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">216
+</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">215
+</t>
+        </is>
+      </c>
+      <c r="N43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">256
+</t>
+        </is>
+      </c>
+      <c r="O43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">990
+</t>
+        </is>
+      </c>
+      <c r="P43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02
+</t>
+        </is>
+      </c>
+      <c r="Q43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">291
+</t>
+        </is>
+      </c>
+      <c r="R43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">255
+</t>
+        </is>
+      </c>
+      <c r="S43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">804
+</t>
+        </is>
+      </c>
+      <c r="T43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">756
+</t>
+        </is>
+      </c>
+      <c r="U43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">98
+</t>
+        </is>
+      </c>
+      <c r="V43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">278
+</t>
+        </is>
+      </c>
+      <c r="W43" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">247
 </t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">87
-</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">198
-</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20
-</t>
-        </is>
-      </c>
-      <c r="J43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">37
-</t>
-        </is>
-      </c>
-      <c r="K43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">00
-</t>
-        </is>
-      </c>
-      <c r="L43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">216
-</t>
-        </is>
-      </c>
-      <c r="M43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">215
-</t>
-        </is>
-      </c>
-      <c r="N43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">256
-</t>
-        </is>
-      </c>
-      <c r="O43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">990
-</t>
-        </is>
-      </c>
-      <c r="P43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">02
-</t>
-        </is>
-      </c>
-      <c r="Q43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">291
-</t>
-        </is>
-      </c>
-      <c r="R43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">255
-</t>
-        </is>
-      </c>
-      <c r="S43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">804
-</t>
-        </is>
-      </c>
-      <c r="T43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">756
-</t>
-        </is>
-      </c>
-      <c r="U43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">98
-</t>
-        </is>
-      </c>
-      <c r="V43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">218
-</t>
-        </is>
-      </c>
-      <c r="W43" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">247
-</t>
-        </is>
-      </c>
       <c r="X43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">291
-</t>
+          <t>341</t>
         </is>
       </c>
       <c r="Y43" s="3" t="inlineStr">
@@ -7013,7 +7017,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">226 1
+          <t xml:space="preserve">226
 </t>
         </is>
       </c>
@@ -7037,7 +7041,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1194
+          <t xml:space="preserve">10494
 </t>
         </is>
       </c>
@@ -7049,7 +7053,7 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">96
+          <t xml:space="preserve">86
 </t>
         </is>
       </c>
@@ -7061,13 +7065,13 @@
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2823
+          <t xml:space="preserve">223
 </t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">823
+          <t xml:space="preserve">223
 </t>
         </is>
       </c>
@@ -7121,7 +7125,7 @@
       </c>
       <c r="V44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">283
+          <t xml:space="preserve">282
 </t>
         </is>
       </c>
@@ -7133,13 +7137,13 @@
       </c>
       <c r="X44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">8282
+          <t xml:space="preserve">322
 </t>
         </is>
       </c>
       <c r="Y44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">844
+          <t xml:space="preserve">1844
 </t>
         </is>
       </c>
@@ -7166,72 +7170,72 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">20262
+          <t xml:space="preserve">2026
 </t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">19016
+          <t xml:space="preserve">1906
 </t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">112986
+          <t xml:space="preserve">11215
 </t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2261
-</t>
+          <t>1563</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">021
+          <t xml:space="preserve">691
 </t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">111 42
+          <t xml:space="preserve">11147
 </t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0110
+          <t xml:space="preserve">1012
 </t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1184
+          <t xml:space="preserve">184
 </t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>7836</t>
+          <t xml:space="preserve">183
+</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11665
+          <t xml:space="preserve">1263
 </t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1239
+          <t xml:space="preserve">101229
 </t>
         </is>
       </c>
       <c r="N45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">11488
+          <t xml:space="preserve">11487
 </t>
         </is>
       </c>
@@ -7261,13 +7265,13 @@
       </c>
       <c r="S45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1211
+          <t xml:space="preserve">1741
 </t>
         </is>
       </c>
       <c r="T45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12300
+          <t xml:space="preserve">24300
 </t>
         </is>
       </c>
@@ -7285,7 +7289,7 @@
       </c>
       <c r="W45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1282
+          <t xml:space="preserve">1449
 </t>
         </is>
       </c>
@@ -7297,12 +7301,13 @@
       </c>
       <c r="Y45" s="3" t="inlineStr">
         <is>
-          <t>5034</t>
+          <t xml:space="preserve">5837
+</t>
         </is>
       </c>
       <c r="Z45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">160
+          <t xml:space="preserve">340
 </t>
         </is>
       </c>
@@ -7329,7 +7334,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1317
+          <t xml:space="preserve">317
 </t>
         </is>
       </c>
@@ -7347,7 +7352,7 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">215
+          <t xml:space="preserve">115
 </t>
         </is>
       </c>
@@ -7369,8 +7374,11 @@
 </t>
         </is>
       </c>
-      <c r="K46" s="3" t="n">
-        <v/>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8
+</t>
+        </is>
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
@@ -7380,7 +7388,7 @@
       </c>
       <c r="M46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">200
+          <t xml:space="preserve">210
 </t>
         </is>
       </c>
@@ -7392,7 +7400,7 @@
       </c>
       <c r="O46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1990
+          <t xml:space="preserve">990
 </t>
         </is>
       </c>
@@ -7404,7 +7412,7 @@
       </c>
       <c r="Q46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">288
+          <t xml:space="preserve">5288
 </t>
         </is>
       </c>
@@ -7422,7 +7430,7 @@
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">229
+          <t xml:space="preserve">750
 </t>
         </is>
       </c>
@@ -7452,13 +7460,14 @@
       </c>
       <c r="Y46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">888
+          <t xml:space="preserve">8239
 </t>
         </is>
       </c>
       <c r="Z46" s="3" t="inlineStr">
         <is>
-          <t>62</t>
+          <t xml:space="preserve">57
+</t>
         </is>
       </c>
       <c r="AA46" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Updated results from latest run in V1.1
</commit_message>
<xml_diff>
--- a/results/01_pre_QA_QC_transcribed_hydroclimate_data/203/203_196905_SF.JPG_pre_QA_QC.xlsx
+++ b/results/01_pre_QA_QC_transcribed_hydroclimate_data/203/203_196905_SF.JPG_pre_QA_QC.xlsx
@@ -949,7 +949,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>1223</t>
+          <t>4223</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="Z8" s="3" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>06</t>
         </is>
       </c>
       <c r="AA8" s="3" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>17835</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="Z9" s="3" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>416</t>
         </is>
       </c>
       <c r="AA9" s="3" t="inlineStr">
@@ -1527,10 +1527,8 @@
           <t>55</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="K10" s="3" t="n">
+        <v/>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
@@ -2474,7 +2472,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
@@ -3129,7 +3127,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>118 2</t>
+          <t>168</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -3154,7 +3152,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>2213</t>
+          <t>213</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
@@ -3732,12 +3730,12 @@
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>282</t>
+          <t>920</t>
         </is>
       </c>
       <c r="U26" s="3" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>20</t>
         </is>
       </c>
       <c r="V26" s="3" t="inlineStr">
@@ -3842,7 +3840,7 @@
       </c>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>1980</t>
+          <t>980</t>
         </is>
       </c>
       <c r="P27" s="3" t="inlineStr">
@@ -3947,7 +3945,7 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
@@ -4262,7 +4260,7 @@
       </c>
       <c r="R30" s="3" t="inlineStr">
         <is>
-          <t>1207 2</t>
+          <t>1207</t>
         </is>
       </c>
       <c r="S30" s="3" t="inlineStr">
@@ -4277,7 +4275,7 @@
       </c>
       <c r="U30" s="3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>105</t>
         </is>
       </c>
       <c r="V30" s="3" t="inlineStr">
@@ -4322,7 +4320,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>2112</t>
+          <t>211</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -4357,7 +4355,7 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>22</t>
         </is>
       </c>
       <c r="K31" s="3" t="n">
@@ -4410,7 +4408,7 @@
       </c>
       <c r="U31" s="3" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>81</t>
         </is>
       </c>
       <c r="V31" s="3" t="inlineStr">
@@ -4960,7 +4958,7 @@
       </c>
       <c r="W35" s="3" t="inlineStr">
         <is>
-          <t>266</t>
+          <t>246</t>
         </is>
       </c>
       <c r="X35" s="3" t="inlineStr">
@@ -5160,7 +5158,7 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>11 01</t>
+          <t>1 01</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -5235,12 +5233,12 @@
       </c>
       <c r="X37" s="3" t="inlineStr">
         <is>
-          <t>1424</t>
+          <t>1824</t>
         </is>
       </c>
       <c r="Y37" s="3" t="inlineStr">
         <is>
-          <t>3922</t>
+          <t>3982</t>
         </is>
       </c>
       <c r="Z37" s="3" t="inlineStr">
@@ -5408,7 +5406,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>2202</t>
+          <t>202</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -5643,7 +5641,7 @@
       </c>
       <c r="Y40" s="3" t="inlineStr">
         <is>
-          <t>720</t>
+          <t>780</t>
         </is>
       </c>
       <c r="Z40" s="3" t="inlineStr">
@@ -6206,7 +6204,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>20262</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -6216,7 +6214,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>1215 2</t>
+          <t>1215</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -6381,7 +6379,7 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>0 1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr">
@@ -6411,7 +6409,7 @@
       </c>
       <c r="Q46" s="3" t="inlineStr">
         <is>
-          <t>2288</t>
+          <t>288</t>
         </is>
       </c>
       <c r="R46" s="3" t="inlineStr">
@@ -6451,7 +6449,7 @@
       </c>
       <c r="Y46" s="3" t="inlineStr">
         <is>
-          <t>832</t>
+          <t>839</t>
         </is>
       </c>
       <c r="Z46" s="3" t="inlineStr">

</xml_diff>